<commit_message>
Final Update for printing receipts
</commit_message>
<xml_diff>
--- a/PromVesClient/Templates/CardTemplate.xlsx
+++ b/PromVesClient/Templates/CardTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Клиент\PromVesClient\PromVesClient\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98F281B9-BE45-4E8C-8A74-CF7B4D71DE8E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E892DDC-73A8-43E5-8867-763974A9883D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,9 +39,6 @@
     <t>Брутто, т.</t>
   </si>
   <si>
-    <t>Грузоподьемность, т.</t>
-  </si>
-  <si>
     <t>Разница бортов, т.</t>
   </si>
   <si>
@@ -64,6 +61,9 @@
   </si>
   <si>
     <t>АО «Уральский завод металлоконструкций»</t>
+  </si>
+  <si>
+    <t>Грузоподъёмность, т.</t>
   </si>
 </sst>
 </file>
@@ -439,7 +439,7 @@
     <col min="5" max="5" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.5703125" customWidth="1"/>
     <col min="7" max="7" width="9.5703125" customWidth="1"/>
-    <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.7109375" customWidth="1"/>
     <col min="9" max="9" width="12.85546875" customWidth="1"/>
     <col min="10" max="10" width="9.28515625" customWidth="1"/>
     <col min="11" max="11" width="10.28515625" customWidth="1"/>
@@ -448,7 +448,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -476,28 +476,28 @@
         <v>2</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>